<commit_message>
n8n board refresh 2026-07-09T17:39:23Z
</commit_message>
<xml_diff>
--- a/app/reports/ARLP_research.xlsx
+++ b/app/reports/ARLP_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-08 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-09 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>49.95</v>
+        <v>50.42</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>24.055</v>
+        <v>24.3596</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.076</v>
+        <v>1.07</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.972</v>
+        <v>0.969</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04577000141143799</v>
+        <v>0.04532999992370605</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>128658799.584286</v>
+        <v>128658800.9655331</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>24.055</v>
+        <v>24.3596</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>3094887424</v>
+        <v>3134076928</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>12.66</v>
+        <v>12.82</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>5.37</v>
+        <v>5.47</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.64</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="6">
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>2757104128</v>
+        <v>2844215296</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>8.189</v>
+        <v>8.265000000000001</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>0.704</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="7">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4107993088</v>
+        <v>4163434752</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>29.808432</v>
+        <v>30.210728</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>11.97</v>
+        <v>11.996</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>2.788</v>
+        <v>2.794</v>
       </c>
     </row>
     <row r="10">
@@ -1638,10 +1638,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>1062070336</v>
+        <v>823709056</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>5.644</v>
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2996305408</v>
+        <v>2962062080</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>29.166668</v>
+        <v>28.833334</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>6.245</v>
+        <v>6.016</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.749</v>
+        <v>1.685</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>1298540416</v>
+        <v>1317284352</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>11.515863</v>
+        <v>11.682091</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.029</v>
+        <v>9.127000000000001</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>6.91</v>
+        <v>6.985</v>
       </c>
     </row>
     <row r="13">

</xml_diff>